<commit_message>
Adding 2035 as a milestone year
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SysSettings.xlsx
+++ b/VerveStacks_EST/SysSettings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40783C0B-64A0-4CE9-82D0-250664437A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D543A72C-41B5-4A95-BC97-55A924E0A464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="system_settings" sheetId="1" r:id="rId1"/>
@@ -4304,7 +4304,7 @@
     </row>
     <row r="16" spans="2:7" ht="15">
       <c r="B16" s="9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>46</v>
@@ -4324,7 +4324,7 @@
     </row>
     <row r="17" spans="2:7" ht="15">
       <c r="B17" s="9">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>46</v>
@@ -4423,7 +4423,9 @@
       </c>
     </row>
     <row r="25" spans="2:7" ht="15">
-      <c r="B25" s="9"/>
+      <c r="B25" s="9">
+        <v>10</v>
+      </c>
       <c r="D25" s="6" t="s">
         <v>46</v>
       </c>

</xml_diff>

<commit_message>
Adding residual file with new commodities
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SysSettings.xlsx
+++ b/VerveStacks_EST/SysSettings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F2336CF-EBAE-4FBA-A74D-B7D9394ACBDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B02C61-5D1A-46DD-BEF8-37FE820AB6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="system_settings" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="281">
   <si>
     <t>~BookRegions_Map</t>
   </si>
@@ -869,6 +869,18 @@
   </si>
   <si>
     <t>PDef1</t>
+  </si>
+  <si>
+    <t>LPG</t>
+  </si>
+  <si>
+    <t>diesel</t>
+  </si>
+  <si>
+    <t>kerosene</t>
+  </si>
+  <si>
+    <t>gasoline</t>
   </si>
 </sst>
 </file>
@@ -3297,6 +3309,9 @@
     <col min="7" max="7" width="13.1796875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="6.7265625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="41.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:18" ht="17.5" thickBot="1">
@@ -3454,7 +3469,7 @@
         <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>21</v>
+        <v>278</v>
       </c>
       <c r="E8" t="s">
         <v>18</v>
@@ -3483,7 +3498,7 @@
         <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
+        <v>279</v>
       </c>
       <c r="E9" t="s">
         <v>18</v>
@@ -3512,7 +3527,7 @@
         <v>17</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>277</v>
       </c>
       <c r="E10" t="s">
         <v>18</v>
@@ -3541,7 +3556,7 @@
         <v>17</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>280</v>
       </c>
       <c r="E11" t="s">
         <v>18</v>
@@ -3570,7 +3585,7 @@
         <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>210</v>
+        <v>21</v>
       </c>
       <c r="E12" t="s">
         <v>18</v>
@@ -3599,10 +3614,19 @@
         <v>17</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E13" t="s">
         <v>18</v>
+      </c>
+      <c r="F13" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" t="s">
+        <v>25</v>
+      </c>
+      <c r="I13" t="s">
+        <v>26</v>
       </c>
       <c r="M13" t="s">
         <v>17</v>
@@ -3628,10 +3652,7 @@
         <v>17</v>
       </c>
       <c r="C14" t="s">
-        <v>204</v>
-      </c>
-      <c r="D14" t="s">
-        <v>206</v>
+        <v>20</v>
       </c>
       <c r="E14" t="s">
         <v>18</v>
@@ -3660,10 +3681,7 @@
         <v>17</v>
       </c>
       <c r="C15" t="s">
-        <v>205</v>
-      </c>
-      <c r="D15" t="s">
-        <v>207</v>
+        <v>23</v>
       </c>
       <c r="E15" t="s">
         <v>18</v>
@@ -3692,23 +3710,11 @@
         <v>17</v>
       </c>
       <c r="C16" t="s">
-        <v>25</v>
-      </c>
-      <c r="D16" t="s">
-        <v>30</v>
+        <v>210</v>
       </c>
       <c r="E16" t="s">
         <v>18</v>
       </c>
-      <c r="F16" t="s">
-        <v>35</v>
-      </c>
-      <c r="G16" t="s">
-        <v>25</v>
-      </c>
-      <c r="I16" t="s">
-        <v>26</v>
-      </c>
       <c r="M16" t="s">
         <v>17</v>
       </c>
@@ -3730,13 +3736,10 @@
     </row>
     <row r="17" spans="2:18">
       <c r="B17" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="C17" t="s">
-        <v>202</v>
-      </c>
-      <c r="D17" t="s">
-        <v>203</v>
+        <v>24</v>
       </c>
       <c r="E17" t="s">
         <v>18</v>
@@ -3762,17 +3765,23 @@
     </row>
     <row r="18" spans="2:18">
       <c r="B18" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>27</v>
+        <v>204</v>
       </c>
       <c r="D18" t="s">
-        <v>31</v>
+        <v>206</v>
       </c>
       <c r="E18" t="s">
         <v>18</v>
       </c>
+      <c r="F18" t="s">
+        <v>35</v>
+      </c>
+      <c r="G18" t="s">
+        <v>25</v>
+      </c>
       <c r="M18" t="s">
         <v>17</v>
       </c>
@@ -3794,13 +3803,13 @@
     </row>
     <row r="19" spans="2:18">
       <c r="B19" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="C19" t="s">
-        <v>28</v>
+        <v>205</v>
       </c>
       <c r="D19" t="s">
-        <v>32</v>
+        <v>207</v>
       </c>
       <c r="E19" t="s">
         <v>18</v>
@@ -3826,13 +3835,13 @@
     </row>
     <row r="20" spans="2:18">
       <c r="B20" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="C20" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D20" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E20" t="s">
         <v>18</v>
@@ -3858,23 +3867,17 @@
     </row>
     <row r="21" spans="2:18">
       <c r="B21" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="C21" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="D21" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="E21" t="s">
         <v>18</v>
       </c>
-      <c r="F21" t="s">
-        <v>35</v>
-      </c>
-      <c r="G21" t="s">
-        <v>25</v>
-      </c>
       <c r="M21" t="s">
         <v>17</v>
       </c>
@@ -3896,16 +3899,16 @@
     </row>
     <row r="22" spans="2:18">
       <c r="B22" t="s">
-        <v>192</v>
+        <v>34</v>
       </c>
       <c r="C22" t="s">
-        <v>193</v>
+        <v>27</v>
       </c>
       <c r="D22" t="s">
-        <v>194</v>
+        <v>31</v>
       </c>
       <c r="E22" t="s">
-        <v>195</v>
+        <v>18</v>
       </c>
       <c r="M22" t="s">
         <v>17</v>
@@ -3928,13 +3931,16 @@
     </row>
     <row r="23" spans="2:18">
       <c r="B23" t="s">
-        <v>192</v>
+        <v>34</v>
       </c>
       <c r="C23" t="s">
-        <v>199</v>
+        <v>28</v>
+      </c>
+      <c r="D23" t="s">
+        <v>32</v>
       </c>
       <c r="E23" t="s">
-        <v>195</v>
+        <v>18</v>
       </c>
       <c r="M23" t="s">
         <v>17</v>
@@ -3957,13 +3963,16 @@
     </row>
     <row r="24" spans="2:18">
       <c r="B24" t="s">
-        <v>192</v>
+        <v>34</v>
       </c>
       <c r="C24" t="s">
-        <v>200</v>
+        <v>29</v>
+      </c>
+      <c r="D24" t="s">
+        <v>33</v>
       </c>
       <c r="E24" t="s">
-        <v>195</v>
+        <v>18</v>
       </c>
       <c r="M24" t="s">
         <v>17</v>
@@ -3985,6 +3994,18 @@
       </c>
     </row>
     <row r="25" spans="2:18">
+      <c r="B25" t="s">
+        <v>17</v>
+      </c>
+      <c r="C25" t="s">
+        <v>196</v>
+      </c>
+      <c r="D25" t="s">
+        <v>197</v>
+      </c>
+      <c r="E25" t="s">
+        <v>18</v>
+      </c>
       <c r="M25" t="s">
         <v>17</v>
       </c>
@@ -4005,6 +4026,18 @@
       </c>
     </row>
     <row r="26" spans="2:18">
+      <c r="B26" t="s">
+        <v>192</v>
+      </c>
+      <c r="C26" t="s">
+        <v>193</v>
+      </c>
+      <c r="D26" t="s">
+        <v>194</v>
+      </c>
+      <c r="E26" t="s">
+        <v>195</v>
+      </c>
       <c r="M26" t="s">
         <v>17</v>
       </c>
@@ -4025,6 +4058,15 @@
       </c>
     </row>
     <row r="27" spans="2:18">
+      <c r="B27" t="s">
+        <v>192</v>
+      </c>
+      <c r="C27" t="s">
+        <v>199</v>
+      </c>
+      <c r="E27" t="s">
+        <v>195</v>
+      </c>
       <c r="M27" t="s">
         <v>17</v>
       </c>
@@ -4045,6 +4087,15 @@
       </c>
     </row>
     <row r="28" spans="2:18">
+      <c r="B28" t="s">
+        <v>192</v>
+      </c>
+      <c r="C28" t="s">
+        <v>200</v>
+      </c>
+      <c r="E28" t="s">
+        <v>195</v>
+      </c>
       <c r="M28" t="s">
         <v>17</v>
       </c>
@@ -4185,8 +4236,8 @@
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C8:C334">
-    <sortCondition ref="C19:C334"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C12:C338">
+    <sortCondition ref="C23:C338"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Correcting file names based on BookName
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SysSettings.xlsx
+++ b/VerveStacks_EST/SysSettings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B02C61-5D1A-46DD-BEF8-37FE820AB6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{717E5AEC-F1E9-4A08-84A6-45EAE2A9EE0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="system_settings" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="281">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="281">
   <si>
     <t>~BookRegions_Map</t>
   </si>
@@ -3231,7 +3231,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:H5"/>
+  <dimension ref="B2:H14"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
@@ -3270,7 +3270,7 @@
     </row>
     <row r="4" spans="2:8">
       <c r="B4" t="s">
-        <v>7</v>
+        <v>212</v>
       </c>
       <c r="C4" t="s">
         <v>212</v>
@@ -3288,6 +3288,14 @@
       </c>
       <c r="H5" t="s">
         <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8">
+      <c r="B14" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" t="s">
+        <v>212</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
guess vervestacks is not that flexible, chanign back syssettings base year to 2022
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SysSettings.xlsx
+++ b/VerveStacks_EST/SysSettings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621948D0-ADC5-4658-A15F-C4300F589B09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51FD8CA6-08AD-4827-A447-86D71D77B8A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -874,7 +874,7 @@
     <t>electricity used in commercial and public sector</t>
   </si>
   <si>
-    <t>msy6_2050</t>
+    <t>msy7_2050</t>
   </si>
 </sst>
 </file>
@@ -4245,7 +4245,7 @@
     </row>
     <row r="4" spans="2:7">
       <c r="B4" s="2">
-        <v>2025</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="7" spans="2:7">
@@ -4275,7 +4275,7 @@
       </c>
       <c r="E12" s="4" t="str">
         <f>"msy"&amp;COUNT(E14:E46)&amp;"_"&amp;MAX(E14:E46)</f>
-        <v>msy7_2053</v>
+        <v>msy7_2050</v>
       </c>
       <c r="F12" s="4" t="str">
         <f>"msy"&amp;COUNT(F14:F45)&amp;"_"&amp;MAX(F14:F45)</f>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="G12" s="4" t="str">
         <f t="shared" ref="G12" si="0">"msy"&amp;COUNT(G14:G45)&amp;"_"&amp;MAX(G14:G45)</f>
-        <v>msy5_2053</v>
+        <v>msy5_2050</v>
       </c>
     </row>
     <row r="13" spans="2:7" ht="15">
@@ -4303,14 +4303,14 @@
       </c>
       <c r="E14" s="2">
         <f>$B$4</f>
-        <v>2025</v>
+        <v>2022</v>
       </c>
       <c r="F14" s="2">
         <v>2025</v>
       </c>
       <c r="G14" s="2">
         <f t="shared" ref="G14" si="1">$B$4</f>
-        <v>2025</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="15" spans="2:7" ht="15">
@@ -4322,14 +4322,14 @@
       </c>
       <c r="E15" s="2">
         <f>E14+3</f>
-        <v>2028</v>
+        <v>2025</v>
       </c>
       <c r="F15" s="2">
         <v>2030</v>
       </c>
       <c r="G15" s="2">
         <f>G14+3</f>
-        <v>2028</v>
+        <v>2025</v>
       </c>
     </row>
     <row r="16" spans="2:7" ht="15">
@@ -4341,14 +4341,14 @@
       </c>
       <c r="E16" s="2">
         <f>E15+5</f>
-        <v>2033</v>
+        <v>2030</v>
       </c>
       <c r="F16" s="2">
         <v>2035</v>
       </c>
       <c r="G16" s="2">
         <f>G15+5</f>
-        <v>2033</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="17" spans="2:7" ht="15">
@@ -4360,14 +4360,14 @@
       </c>
       <c r="E17" s="2">
         <f t="shared" ref="E17:E20" si="2">E16+5</f>
-        <v>2038</v>
+        <v>2035</v>
       </c>
       <c r="F17" s="2">
         <v>2040</v>
       </c>
       <c r="G17" s="2">
         <f>G16+10</f>
-        <v>2043</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="18" spans="2:7" ht="15">
@@ -4379,14 +4379,14 @@
       </c>
       <c r="E18" s="2">
         <f t="shared" si="2"/>
-        <v>2043</v>
+        <v>2040</v>
       </c>
       <c r="F18" s="2">
         <v>2045</v>
       </c>
       <c r="G18" s="2">
         <f t="shared" ref="G18" si="3">G17+10</f>
-        <v>2053</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="19" spans="2:7" ht="15">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="E19" s="2">
         <f t="shared" si="2"/>
-        <v>2048</v>
+        <v>2045</v>
       </c>
       <c r="F19" s="2">
         <v>2050</v>
@@ -4411,7 +4411,7 @@
       </c>
       <c r="E20" s="2">
         <f t="shared" si="2"/>
-        <v>2053</v>
+        <v>2050</v>
       </c>
     </row>
     <row r="21" spans="2:7" ht="15">

</xml_diff>

<commit_message>
Taking syssettings from dev
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SysSettings.xlsx
+++ b/VerveStacks_EST/SysSettings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51FD8CA6-08AD-4827-A447-86D71D77B8A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69A338A-4A0E-4102-A22D-C3DD5E06221D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="system_settings" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="279">
   <si>
     <t>~BookRegions_Map</t>
   </si>
@@ -1279,6 +1279,8 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="186"/>
     </font>
   </fonts>
   <fills count="47">
@@ -3311,7 +3313,7 @@
   <cols>
     <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="44.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="3.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
@@ -3856,6 +3858,9 @@
       </c>
       <c r="D20" t="s">
         <v>277</v>
+      </c>
+      <c r="E20" t="s">
+        <v>18</v>
       </c>
       <c r="M20" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
Adding grid nodes to SysSettings.xlsx
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SysSettings.xlsx
+++ b/VerveStacks_EST/SysSettings.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E69A338A-4A0E-4102-A22D-C3DD5E06221D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C2974C9-9781-4AAA-9F5C-D7612F249764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="system_settings" sheetId="1" r:id="rId1"/>
     <sheet name="fuels" sheetId="2" r:id="rId2"/>
-    <sheet name="TimePeriods" sheetId="3" r:id="rId3"/>
-    <sheet name="System Settings" sheetId="4" r:id="rId4"/>
-    <sheet name="Constants" sheetId="5" r:id="rId5"/>
-    <sheet name="reporting options" sheetId="6" r:id="rId6"/>
+    <sheet name="grids" sheetId="7" r:id="rId3"/>
+    <sheet name="TimePeriods" sheetId="3" r:id="rId4"/>
+    <sheet name="System Settings" sheetId="4" r:id="rId5"/>
+    <sheet name="Constants" sheetId="5" r:id="rId6"/>
+    <sheet name="reporting options" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="311">
   <si>
     <t>~BookRegions_Map</t>
   </si>
@@ -875,6 +876,102 @@
   </si>
   <si>
     <t>msy7_2050</t>
+  </si>
+  <si>
+    <t>e_harku_330</t>
+  </si>
+  <si>
+    <t>Harku alajaam</t>
+  </si>
+  <si>
+    <t>lo</t>
+  </si>
+  <si>
+    <t>e_pussi_330</t>
+  </si>
+  <si>
+    <t>Pussi alajaam</t>
+  </si>
+  <si>
+    <t>e_kilingi_nomme_330</t>
+  </si>
+  <si>
+    <t>Killingi-Nomme alajaam</t>
+  </si>
+  <si>
+    <t>e_tsirguliina_330</t>
+  </si>
+  <si>
+    <t>Tsirguliina alajaam</t>
+  </si>
+  <si>
+    <t>e_tartu_330</t>
+  </si>
+  <si>
+    <t>Tartu alajaam</t>
+  </si>
+  <si>
+    <t>e_arukula_330</t>
+  </si>
+  <si>
+    <t>Arukula alajaam</t>
+  </si>
+  <si>
+    <t>e_baltiej_330</t>
+  </si>
+  <si>
+    <t>Balti EJ alajaam</t>
+  </si>
+  <si>
+    <t>e_viru_330</t>
+  </si>
+  <si>
+    <t>Viru alajaam</t>
+  </si>
+  <si>
+    <t>e_kiisa_330</t>
+  </si>
+  <si>
+    <t>Kiisa alajaam</t>
+  </si>
+  <si>
+    <t>e_paide_330</t>
+  </si>
+  <si>
+    <t>Paide alajaam</t>
+  </si>
+  <si>
+    <t>e_sopi_330</t>
+  </si>
+  <si>
+    <t>Sopi alajaam</t>
+  </si>
+  <si>
+    <t>e_sindi_330</t>
+  </si>
+  <si>
+    <t>Sindi alajaam</t>
+  </si>
+  <si>
+    <t>e_mustvee_330</t>
+  </si>
+  <si>
+    <t>Mustvee alajaam</t>
+  </si>
+  <si>
+    <t>e_rakvere_330</t>
+  </si>
+  <si>
+    <t>Rakvere alajaam</t>
+  </si>
+  <si>
+    <t>e_lihula_330</t>
+  </si>
+  <si>
+    <t>Lihula alajaam</t>
+  </si>
+  <si>
+    <t>~fi_comm</t>
   </si>
 </sst>
 </file>
@@ -4230,6 +4327,393 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8CD4434-6BD0-409F-A92E-16A0D49E7A83}">
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>279</v>
+      </c>
+      <c r="C3" t="s">
+        <v>280</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" t="s">
+        <v>281</v>
+      </c>
+      <c r="G3" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>282</v>
+      </c>
+      <c r="C4" t="s">
+        <v>283</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" t="s">
+        <v>281</v>
+      </c>
+      <c r="G4" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" t="s">
+        <v>284</v>
+      </c>
+      <c r="C5" t="s">
+        <v>285</v>
+      </c>
+      <c r="D5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" t="s">
+        <v>281</v>
+      </c>
+      <c r="G5" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>286</v>
+      </c>
+      <c r="C6" t="s">
+        <v>287</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F6" t="s">
+        <v>281</v>
+      </c>
+      <c r="G6" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>288</v>
+      </c>
+      <c r="C7" t="s">
+        <v>289</v>
+      </c>
+      <c r="D7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" t="s">
+        <v>281</v>
+      </c>
+      <c r="G7" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C8" t="s">
+        <v>291</v>
+      </c>
+      <c r="D8" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" t="s">
+        <v>281</v>
+      </c>
+      <c r="G8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>292</v>
+      </c>
+      <c r="C9" t="s">
+        <v>293</v>
+      </c>
+      <c r="D9" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" t="s">
+        <v>281</v>
+      </c>
+      <c r="G9" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" t="s">
+        <v>294</v>
+      </c>
+      <c r="C10" t="s">
+        <v>295</v>
+      </c>
+      <c r="D10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" t="s">
+        <v>35</v>
+      </c>
+      <c r="F10" t="s">
+        <v>281</v>
+      </c>
+      <c r="G10" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" t="s">
+        <v>296</v>
+      </c>
+      <c r="C11" t="s">
+        <v>297</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" t="s">
+        <v>35</v>
+      </c>
+      <c r="F11" t="s">
+        <v>281</v>
+      </c>
+      <c r="G11" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" t="s">
+        <v>298</v>
+      </c>
+      <c r="C12" t="s">
+        <v>299</v>
+      </c>
+      <c r="D12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" t="s">
+        <v>281</v>
+      </c>
+      <c r="G12" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" t="s">
+        <v>300</v>
+      </c>
+      <c r="C13" t="s">
+        <v>301</v>
+      </c>
+      <c r="D13" t="s">
+        <v>25</v>
+      </c>
+      <c r="E13" t="s">
+        <v>35</v>
+      </c>
+      <c r="F13" t="s">
+        <v>281</v>
+      </c>
+      <c r="G13" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>302</v>
+      </c>
+      <c r="C14" t="s">
+        <v>303</v>
+      </c>
+      <c r="D14" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" t="s">
+        <v>35</v>
+      </c>
+      <c r="F14" t="s">
+        <v>281</v>
+      </c>
+      <c r="G14" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" t="s">
+        <v>304</v>
+      </c>
+      <c r="C15" t="s">
+        <v>305</v>
+      </c>
+      <c r="D15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E15" t="s">
+        <v>35</v>
+      </c>
+      <c r="F15" t="s">
+        <v>281</v>
+      </c>
+      <c r="G15" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>306</v>
+      </c>
+      <c r="C16" t="s">
+        <v>307</v>
+      </c>
+      <c r="D16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" t="s">
+        <v>35</v>
+      </c>
+      <c r="F16" t="s">
+        <v>281</v>
+      </c>
+      <c r="G16" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" t="s">
+        <v>308</v>
+      </c>
+      <c r="C17" t="s">
+        <v>309</v>
+      </c>
+      <c r="D17" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" t="s">
+        <v>35</v>
+      </c>
+      <c r="F17" t="s">
+        <v>281</v>
+      </c>
+      <c r="G17" t="s">
+        <v>216</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A39735C-B147-4873-BE33-BF7570891F36}">
   <dimension ref="B3:G33"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
@@ -4491,7 +4975,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A64C410-895F-4040-A7AB-3F7211AA7FBD}">
   <dimension ref="B1:N42"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12"/>
@@ -5072,7 +5556,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5EBD23C-EA82-4040-97D7-F532F0547462}">
   <dimension ref="A2:N102"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12"/>
@@ -6712,7 +7196,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DE1F0D2-7682-484B-9627-54FDDA96E26C}">
   <dimension ref="B3:D33"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="12.75"/>

</xml_diff>

<commit_message>
Adding costs to export from Estlinks
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SysSettings.xlsx
+++ b/VerveStacks_EST/SysSettings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7901D393-71BC-4F76-843F-C7CFF15B21B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{407DA071-CE15-478A-955B-B7C199FDA722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="system_settings" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="706" uniqueCount="274">
   <si>
     <t>~BookRegions_Map</t>
   </si>
@@ -857,6 +857,9 @@
   </si>
   <si>
     <t>elv_spv_hiiu</t>
+  </si>
+  <si>
+    <t>EUR25</t>
   </si>
 </sst>
 </file>
@@ -5049,7 +5052,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5EBD23C-EA82-4040-97D7-F532F0547462}">
-  <dimension ref="A2:N102"/>
+  <dimension ref="A2:N104"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="7"/>
@@ -6681,6 +6684,31 @@
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
+    <row r="103" spans="5:10">
+      <c r="F103" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="H103" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="I103" s="7">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="104" spans="5:10">
+      <c r="F104" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="G104" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="H104" s="7" t="s">
+        <v>273</v>
+      </c>
+      <c r="I104" s="7">
+        <v>1.33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Adding interp rule for flo_fr
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SysSettings.xlsx
+++ b/VerveStacks_EST/SysSettings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F3135F5-49E9-4A94-8864-5F757430CA5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9863DA41-8A5E-42BE-B190-F410B134209D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="system_settings" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="707" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="275">
   <si>
     <t>~BookRegions_Map</t>
   </si>
@@ -860,6 +860,9 @@
   </si>
   <si>
     <t>elc_spv_hiiu</t>
+  </si>
+  <si>
+    <t>flo_fr</t>
   </si>
 </sst>
 </file>
@@ -4624,6 +4627,17 @@
         <v>3</v>
       </c>
     </row>
+    <row r="12" spans="2:12">
+      <c r="D12" s="7" t="s">
+        <v>274</v>
+      </c>
+      <c r="E12" s="7">
+        <v>0</v>
+      </c>
+      <c r="F12" s="7">
+        <v>5</v>
+      </c>
+    </row>
     <row r="14" spans="2:12">
       <c r="B14" s="10" t="s">
         <v>62</v>

</xml_diff>